<commit_message>
elite and elevate CC issued.
</commit_message>
<xml_diff>
--- a/frontend/Premium Final Submission Form (Responses).xlsx
+++ b/frontend/Premium Final Submission Form (Responses).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal\internship_portal\frontend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5DDADE4-7A2F-44F7-AAC9-2A2D67274853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0F32F3A-F8DE-49A8-BC5D-56FF3933F929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C47EE7DD-172B-4A1B-B9E4-8FA1669923F8}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="175">
   <si>
     <t xml:space="preserve">Full Name </t>
   </si>
@@ -344,13 +344,214 @@
   </si>
   <si>
     <t xml:space="preserve"> 26T-A-WD</t>
+  </si>
+  <si>
+    <t>kavya ramadoss</t>
+  </si>
+  <si>
+    <t>S.K.Hariaharan</t>
+  </si>
+  <si>
+    <t>J DIPTO JAISON</t>
+  </si>
+  <si>
+    <t>Akash kumar V</t>
+  </si>
+  <si>
+    <t>S JEGATHISAN</t>
+  </si>
+  <si>
+    <t>Vishva.M</t>
+  </si>
+  <si>
+    <t>Harthe.R</t>
+  </si>
+  <si>
+    <t>Y. BESCHI ANTO</t>
+  </si>
+  <si>
+    <t>Prasanna.K</t>
+  </si>
+  <si>
+    <t>YOGESH KUMAR M</t>
+  </si>
+  <si>
+    <t>Girishkumar M</t>
+  </si>
+  <si>
+    <t>M26IP141</t>
+  </si>
+  <si>
+    <t>M26IP134</t>
+  </si>
+  <si>
+    <t>M26IP139</t>
+  </si>
+  <si>
+    <t>ID:M26IP281</t>
+  </si>
+  <si>
+    <t>M261P199</t>
+  </si>
+  <si>
+    <t>M26IP078</t>
+  </si>
+  <si>
+    <t>M26IP116</t>
+  </si>
+  <si>
+    <t>M26IP007</t>
+  </si>
+  <si>
+    <t>M26IP008</t>
+  </si>
+  <si>
+    <t>M26IP279</t>
+  </si>
+  <si>
+    <t>M26IP003</t>
+  </si>
+  <si>
+    <t>Web development fundamentals</t>
+  </si>
+  <si>
+    <t>Web development fundam</t>
+  </si>
+  <si>
+    <t>Frontend development (HTML &amp; CSS)</t>
+  </si>
+  <si>
+    <t>Medical device fundamentals</t>
+  </si>
+  <si>
+    <t>Entrepreneurship Fundamentals</t>
+  </si>
+  <si>
+    <t>Frontend development</t>
+  </si>
+  <si>
+    <t>26T-J-MD</t>
+  </si>
+  <si>
+    <t>26NT-C-ENT</t>
+  </si>
+  <si>
+    <t>N. ARUN KUMAR</t>
+  </si>
+  <si>
+    <t>KARTHIKEYAN E</t>
+  </si>
+  <si>
+    <t>Lourdu Flavin Romaro B</t>
+  </si>
+  <si>
+    <t>S. Vyash</t>
+  </si>
+  <si>
+    <t>A.Vignesh</t>
+  </si>
+  <si>
+    <t>J.Priyadharshini</t>
+  </si>
+  <si>
+    <t>A. Krishnamoorthy</t>
+  </si>
+  <si>
+    <t>Birundha C</t>
+  </si>
+  <si>
+    <t>KISHORE M</t>
+  </si>
+  <si>
+    <t>KABILAN.M</t>
+  </si>
+  <si>
+    <t>Krishnaraj M</t>
+  </si>
+  <si>
+    <t>Logeshwaran S</t>
+  </si>
+  <si>
+    <t>Syed Saifuddin</t>
+  </si>
+  <si>
+    <t>Santhosh. D</t>
+  </si>
+  <si>
+    <t>Dharsan</t>
+  </si>
+  <si>
+    <t>M26IP275</t>
+  </si>
+  <si>
+    <t>M26IP80</t>
+  </si>
+  <si>
+    <t>M26IP269</t>
+  </si>
+  <si>
+    <t>M26IP268</t>
+  </si>
+  <si>
+    <t>M26IP283</t>
+  </si>
+  <si>
+    <t>M26IP273</t>
+  </si>
+  <si>
+    <t>M26IP274</t>
+  </si>
+  <si>
+    <t>M26IP289</t>
+  </si>
+  <si>
+    <t>M26IP290</t>
+  </si>
+  <si>
+    <t>M26IP292</t>
+  </si>
+  <si>
+    <t>M26IP294</t>
+  </si>
+  <si>
+    <t>M26IP271</t>
+  </si>
+  <si>
+    <t>M26IP282</t>
+  </si>
+  <si>
+    <t>M26IP291</t>
+  </si>
+  <si>
+    <t>M26IP266</t>
+  </si>
+  <si>
+    <t>Digital marketing</t>
+  </si>
+  <si>
+    <t>Frontend development (html and CSS)</t>
+  </si>
+  <si>
+    <t>UI/UX development</t>
+  </si>
+  <si>
+    <t>Web development and fundamentals</t>
+  </si>
+  <si>
+    <t>Java programming</t>
+  </si>
+  <si>
+    <t>26T-B-UID</t>
+  </si>
+  <si>
+    <t>Elevate</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -485,8 +686,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF434343"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Roboto"/>
+    </font>
   </fonts>
-  <fills count="35">
+  <fills count="37">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -678,8 +889,20 @@
         <bgColor rgb="FFF8F9FA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8F9FA"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="11">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -809,6 +1032,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -854,7 +1099,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -868,14 +1113,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1232,7 +1495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EC2C977-6593-425B-AEB9-E3A7F18DC4A2}">
-  <dimension ref="B1:AB34"/>
+  <dimension ref="B1:AB64"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" customWidth="1"/>
@@ -1620,10 +1883,10 @@
       <c r="E21" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="G21" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1640,10 +1903,10 @@
       <c r="E22" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G22" s="7" t="s">
+      <c r="G22" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1660,10 +1923,10 @@
       <c r="E23" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G23" s="7" t="s">
+      <c r="G23" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1680,10 +1943,10 @@
       <c r="E24" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="F24" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="G24" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1700,10 +1963,10 @@
       <c r="E25" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="F25" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G25" s="7" t="s">
+      <c r="G25" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1720,10 +1983,10 @@
       <c r="E26" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="F26" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G26" s="7" t="s">
+      <c r="G26" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1740,10 +2003,10 @@
       <c r="E27" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="F27" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G27" s="7" t="s">
+      <c r="G27" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1760,10 +2023,10 @@
       <c r="E28" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G28" s="7" t="s">
+      <c r="G28" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1780,10 +2043,10 @@
       <c r="E29" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F29" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="G29" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1800,10 +2063,10 @@
       <c r="E30" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="F30" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G30" s="7" t="s">
+      <c r="G30" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1820,10 +2083,10 @@
       <c r="E31" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="F31" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G31" s="7" t="s">
+      <c r="G31" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1840,10 +2103,10 @@
       <c r="E32" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="F32" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G32" s="7" t="s">
+      <c r="G32" s="3" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1860,32 +2123,556 @@
       <c r="E33" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="F33" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="G33" s="7" t="s">
+      <c r="G33" s="3" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="34" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B34" s="6" t="s">
+      <c r="B34" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="D34" s="6" t="s">
+      <c r="D34" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="E34" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="F34" s="8" t="s">
         <v>106</v>
       </c>
-      <c r="G34" s="7" t="s">
-        <v>55</v>
-      </c>
+      <c r="G34" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="35" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B35" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="36" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B36" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C36" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="D36" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="E36" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="37" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B37" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="D37" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="E37" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="38" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B38" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C38" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="D38" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E38" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="39" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B39" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="D39" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="E39" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="40" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B40" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C40" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="D40" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E40" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="41" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B41" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="42" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B42" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C42" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="D42" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="E42" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="43" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B43" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F43" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G43" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="44" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B44" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C44" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="D44" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F44" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="45" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B45" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="E45" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="F45" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B49" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="C49" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F49" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="50" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B50" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="C50" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E50" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="51" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B51" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B52" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="C52" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="D52" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="E52" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B53" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B54" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="C54" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="D54" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="E54" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="F54" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G54" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B55" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F55" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G55" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B56" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="D56" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="E56" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G56" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="57" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B57" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E57" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G57" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="58" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B58" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="C58" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="D58" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F58" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G58" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="59" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B59" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="E59" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F59" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G59" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="60" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B60" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="C60" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="D60" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="E60" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F60" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G60" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="61" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B61" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="C61" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="D61" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F61" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G61" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="62" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B62" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="C62" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="D62" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="E62" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F62" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G62" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="63" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B63" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="C63" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="D63" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="E63" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F63" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G63" s="9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="F64" s="13"/>
+      <c r="G64" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>